<commit_message>
fix: trace NMDB performance definitions and gaps
</commit_message>
<xml_diff>
--- a/apps/excel/templates/CreditAtlas-NMDB-Performance.xlsx
+++ b/apps/excel/templates/CreditAtlas-NMDB-Performance.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bat dau" sheetId="1" r:id="Ra6349c4b1bf34942"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Latest KPIs" sheetId="2" r:id="R4aae4000769448b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly data" sheetId="3" r:id="Rf9f89328377b4e90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definitions" sheetId="4" r:id="Rea246f7dad914cc1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bat dau" sheetId="1" r:id="Re6de2cf4d49443ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Latest KPIs" sheetId="2" r:id="Rccc0d65e385149b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly data" sheetId="3" r:id="Rf1666f2252ac45e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definitions" sheetId="4" r:id="R787dfae427884b64"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -158,7 +158,7 @@
     <x:tableColumn id="1" name="Quarter"/>
     <x:tableColumn id="2" name="Mortgage market"/>
     <x:tableColumn id="3" name="Publisher market definition"/>
-    <x:tableColumn id="4" name="30–60 DPD (%)"/>
+    <x:tableColumn id="4" name="30–89 DPD (%)"/>
     <x:tableColumn id="5" name="90+ DPD (%)"/>
     <x:tableColumn id="6" name="Foreclosure / bankruptcy / DIL (%)"/>
     <x:tableColumn id="7" name="Forbearance (%)"/>
@@ -460,7 +460,7 @@
         <x:v>Thận trọng</x:v>
       </x:c>
       <x:c r="B8" s="8" t="str">
-        <x:v>Hai quý mới nhất là sơ bộ; xem Definitions về active-loan mẫu số, stale-account rule, reporting lag và giới hạn 2006–2012.</x:v>
+        <x:v>Hai quý mới nhất là sơ bộ; P3089DL gộp nhóm 30–59 và 60–89 ngày quá hạn; xem Definitions về mẫu số, stale-account rule, reporting lag và giới hạn 2006–2012.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -503,7 +503,7 @@
         <x:v>Publisher market definition</x:v>
       </x:c>
       <x:c r="D1" s="12" t="str">
-        <x:v>30–60 DPD (%)</x:v>
+        <x:v>30–89 DPD (%)</x:v>
       </x:c>
       <x:c r="E1" s="12" t="str">
         <x:v>90+ DPD (%)</x:v>
@@ -610,7 +610,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R235029b9b2a84886"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a5820c72b8d4c54"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -64398,7 +64398,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb57eca4baa14459c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51ccd7f0fc9744bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -64432,13 +64432,13 @@
         <x:v>P3089DL</x:v>
       </x:c>
       <x:c r="B2" s="13" t="str">
-        <x:v>30–60 days past due</x:v>
+        <x:v>30–89 days delinquent</x:v>
       </x:c>
       <x:c r="C2" s="13" t="str">
-        <x:v>Active loans at least 30 or 60 days past due divided by all active loans at quarter end.</x:v>
+        <x:v>Active loans in either FHFA 30–59 or 60–89 days-past-due category divided by all active loans at quarter end. FHFA combines the source categories in P3089DL.</x:v>
       </x:c>
       <x:c r="D2" s="13" t="str">
-        <x:v>Quarter-end performance category.</x:v>
+        <x:v>Quarter-end performance category; use the readable label 30–89 DPD.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -64570,7 +64570,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree3f2b572eba465a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4280de724777487a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>